<commit_message>
Correct formal errors in second coding (K-10)
</commit_message>
<xml_diff>
--- a/kodierung/zweitkodierung/kodiertabelle_zweit.xlsx
+++ b/kodierung/zweitkodierung/kodiertabelle_zweit.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="730" uniqueCount="243">
   <si>
     <t>kodier_id</t>
   </si>
@@ -35,12 +35,12 @@
     <t>kb_abdeckung</t>
   </si>
   <si>
+    <t>K1–K3</t>
+  </si>
+  <si>
     <t>schwierigkeit</t>
   </si>
   <si>
-    <t>K1–K3</t>
-  </si>
-  <si>
     <t>K1</t>
   </si>
   <si>
@@ -50,63 +50,63 @@
     <t>Freitext</t>
   </si>
   <si>
+    <t>vorgegeben aus der Erstkodierung (K-06), blau hinterlegt, nicht ändern; leer, wenn die Erstkodierung keine Kernaussage festgestellt hat</t>
+  </si>
+  <si>
     <t>K1_C2</t>
   </si>
   <si>
-    <t>vorgegeben aus der Erstkodierung (K-06), blau hinterlegt, nicht ändern; leer, wenn die Erstkodierung keine Kernaussage festgestellt hat</t>
+    <t>Kx_C1</t>
+  </si>
+  <si>
+    <t>gedeckt / teilweise / nicht gedeckt</t>
   </si>
   <si>
     <t>K2</t>
   </si>
   <si>
-    <t>Kx_C1</t>
-  </si>
-  <si>
-    <t>gedeckt / teilweise / nicht gedeckt</t>
+    <t>Ist die Kernaussage durch die gesamte KB gedeckt?</t>
+  </si>
+  <si>
+    <t>Kx_C2</t>
+  </si>
+  <si>
+    <t>passend / nicht passend / kein Beleg</t>
   </si>
   <si>
     <t>K2_C1</t>
   </si>
   <si>
-    <t>Ist die Kernaussage durch die gesamte KB gedeckt?</t>
+    <t>Stützt der im Satz angegebene Beleg die Aussage? LLM-only: immer „kein Beleg“</t>
   </si>
   <si>
     <t>K2_C2</t>
   </si>
   <si>
-    <t>Kx_C2</t>
-  </si>
-  <si>
-    <t>passend / nicht passend / kein Beleg</t>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>ja / nein</t>
   </si>
   <si>
     <t>K3</t>
   </si>
   <si>
-    <t>Stützt der im Satz angegebene Beleg die Aussage? LLM-only: immer „kein Beleg“</t>
+    <t>Tritt eine Rückfrage, Enthaltung oder Weiterleitung an die Stelle einer Sachaussage zu einem Anliegen?</t>
+  </si>
+  <si>
+    <t>mangel</t>
   </si>
   <si>
     <t>K3_C1</t>
   </si>
   <si>
-    <t>C3</t>
-  </si>
-  <si>
-    <t>ja / nein</t>
-  </si>
-  <si>
-    <t>Tritt eine Rückfrage, Enthaltung oder Weiterleitung an die Stelle einer Sachaussage zu einem Anliegen?</t>
+    <t>Nur RAG: ungedeckte Aussage, unbeantwortetes Anliegen (KB-gedeckt) oder Belegproblem?</t>
   </si>
   <si>
     <t>K3_C2</t>
   </si>
   <si>
-    <t>mangel</t>
-  </si>
-  <si>
-    <t>Nur RAG: ungedeckte Aussage, unbeantwortetes Anliegen (KB-gedeckt) oder Belegproblem?</t>
-  </si>
-  <si>
     <t>F_primaer</t>
   </si>
   <si>
@@ -122,18 +122,18 @@
     <t>z. B. F3;F4</t>
   </si>
   <si>
+    <t>weitere zutreffende Typen, mit Semikolon getrennt</t>
+  </si>
+  <si>
     <t>bemerkung</t>
   </si>
   <si>
-    <t>weitere zutreffende Typen, mit Semikolon getrennt</t>
+    <t>Begründung bei Unsicherheit oder Mischfall</t>
   </si>
   <si>
     <t>K012</t>
   </si>
   <si>
-    <t>Begründung bei Unsicherheit oder Mischfall</t>
-  </si>
-  <si>
     <t>T-120</t>
   </si>
   <si>
@@ -365,301 +365,304 @@
     <t>Rücktransport der Speditionsware fallen Kosten in Höhe von 49 € an, die von der Erstattung abgezogen werden. Die Ware muss zerlegt und abholbereit im Erdgeschoss bereitgestellt werden</t>
   </si>
   <si>
+    <t>Fehlerhafte Ware wurde nicht berücksichtigt</t>
+  </si>
+  <si>
+    <t>K074</t>
+  </si>
+  <si>
+    <t>T-040</t>
+  </si>
+  <si>
+    <t>eine Rücksendung ist auch ohne die Originalverpackung möglich, da diese zwar erwünscht, aber nicht verpflichtend ist</t>
+  </si>
+  <si>
+    <t>melden Sie die Rücksendung über das Retourenportal in Ihrem Kundenkonto an oder als Gast mit Bestellnummer und Postleitzahl.</t>
+  </si>
+  <si>
+    <t>Sollte es sich um eine Maßanfertigung handeln, ist eine Rückgabe ausgeschlossen</t>
+  </si>
+  <si>
+    <t>K077</t>
+  </si>
+  <si>
+    <t>T-090</t>
+  </si>
+  <si>
+    <t>Eine Verlängerung der Garantiezeit auf 10 Jahre, auch gegen Aufpreis, ist bei uns derzeit nicht vorgesehen.</t>
+  </si>
+  <si>
+    <t>K078</t>
+  </si>
+  <si>
+    <t>T-011</t>
+  </si>
+  <si>
+    <t>Grundsätzlich bieten wir die Möglichkeit, Lieferungen an Packstationen zu senden, sofern dies vom Versanddienstleister unterstützt wird</t>
+  </si>
+  <si>
+    <t>K088</t>
+  </si>
+  <si>
+    <t>T-067</t>
+  </si>
+  <si>
+    <t>für Möbel der Eigenmarke HD Basics, wie Ihr Regal, erhalten Sie eine 5-Jahres-Herstellergarantie</t>
+  </si>
+  <si>
+    <t>Eine Registrierung des Produkts ist nicht erforderlich. Ihre Rechnung dient als Nachweis für die Garantie</t>
+  </si>
+  <si>
+    <t>K091</t>
+  </si>
+  <si>
+    <t>T-083</t>
+  </si>
+  <si>
+    <t>Bitte melden Sie den Schaden möglichst schnell, idealerweise mit Fotos, damit wir den Fall besser prüfen können. Sie können uns die Fotos gerne per E-Mail oder über das Kontaktformular auf unserer Webseite senden</t>
+  </si>
+  <si>
+    <t>Bezüglich der weiteren Vorgehensweise können wir Ihnen nach Prüfung des Schadens verschiedene Optionen anbieten, wie Ersatzlieferung oder Rückerstattung</t>
+  </si>
+  <si>
+    <t>K099</t>
+  </si>
+  <si>
+    <t>T-104</t>
+  </si>
+  <si>
+    <t>Leider können wir aus Datenschutz- und Sicherheitsgründen keine genauen Gründe für die Ablehnung nennen. Möglicherweise hängt dies mit internen Prüfungen oder Bonitätsbewertungen zusammen.</t>
+  </si>
+  <si>
+    <t>Alternativ bieten wir Ihnen verschiedene andere Zahlungsmöglichkeiten an, wie zum Beispiel Kreditkarte, PayPal oder Vorkasse.</t>
+  </si>
+  <si>
+    <t>K101</t>
+  </si>
+  <si>
+    <t>T-043</t>
+  </si>
+  <si>
+    <t>Rückgabe von Speditionsware in Österreich müssen Sie die Retoure innerhalb von 14 Tagen ab Erhalt der Ware über unseren Kundenservice anmelden</t>
+  </si>
+  <si>
+    <t>vereinbaren Sie bitte einen Abholtermin mit der Spedition. Die Ware muss zerlegt und abholbereit im Erdgeschoss bereitgestellt werden</t>
+  </si>
+  <si>
+    <t>Rücktransportkosten für Speditionsware in Österreich betragen 69 Euro und werden von der Erstattung abgezogen</t>
+  </si>
+  <si>
+    <t>K115</t>
+  </si>
+  <si>
+    <t>K117</t>
+  </si>
+  <si>
+    <t>T-060</t>
+  </si>
+  <si>
+    <t>In der Regel versenden wir Retourenlabels per E-Mail zum Ausdrucken</t>
+  </si>
+  <si>
+    <t>Wenn Sie keinen Drucker zur Verfügung haben, prüfen wir gerne, ob wir Ihnen das Retourenlabel auch per Post zusenden können</t>
+  </si>
+  <si>
+    <t>K123</t>
+  </si>
+  <si>
+    <t>T-042</t>
+  </si>
+  <si>
+    <t>eine Rückgabe von Speditionsware ist grundsätzlich innerhalb von 14 Tagen ab Erhalt möglich; weil 20 Tage nicht mehr möglich</t>
+  </si>
+  <si>
+    <t>Anmeldung einer Rücksendung von Speditionsware ist eine Kontaktaufnahme mit unserem Kundenservice innerhalb der Widerrufsfrist erforderlich. Die Rückgabe erfolgt ausschließlich über den Kundenservice, nicht über das Retourenportal</t>
+  </si>
+  <si>
+    <t>F3</t>
+  </si>
+  <si>
+    <t>Widerruf verstrichen</t>
+  </si>
+  <si>
+    <t>K127</t>
+  </si>
+  <si>
+    <t>T-088</t>
+  </si>
+  <si>
+    <t>K129</t>
+  </si>
+  <si>
+    <t>T-105</t>
+  </si>
+  <si>
+    <t>Grundsätzlich können Geschenkgutscheine von Hallendal Wohnen auch für Bestellungen aus der Schweiz eingelöst werden</t>
+  </si>
+  <si>
+    <t>Bezüglich der Zahlungsmöglichkeiten für Kunden aus der Schweiz bieten wir verschiedene Optionen an</t>
+  </si>
+  <si>
+    <t>K136</t>
+  </si>
+  <si>
+    <t>T-094</t>
+  </si>
+  <si>
+    <t>der Kauf auf Rechnung ist bei Hallendal Wohnen nur bis zu einem maximalen Bestellwert von 1.500 Euro möglich</t>
+  </si>
+  <si>
+    <t>K156</t>
+  </si>
+  <si>
+    <t>Grundsätzlich haben Sie das Recht, Ihre Bestellung innerhalb von 14 Tagen nach Erhalt zurückzugeben.</t>
+  </si>
+  <si>
+    <t>Bezüglich der Erstattung der Versandkosten für den Hinweg hängt dies von den jeweiligen Bedingungen ab, die in unseren Rückgabebedingungen geregelt sind.</t>
+  </si>
+  <si>
+    <t>K159</t>
+  </si>
+  <si>
+    <t>T-080</t>
+  </si>
+  <si>
+    <t>5-Jahres-Herstellergarantie, die ab Lieferung gilt; Das durchgesessene Polster im Kopfteil fällt daher nicht unter die Garantie</t>
+  </si>
+  <si>
+    <t>Für das defekte Teil der Halterung können Sie sich gerne an unseren Kundenservice wenden und die Artikelnummer Ihres Bettes angeben.</t>
+  </si>
+  <si>
+    <t>Montageanleitungen finden Sie als PDF auf der Produktseite Ihres Bettes.</t>
+  </si>
+  <si>
+    <t>K166</t>
+  </si>
+  <si>
+    <t>T-032</t>
+  </si>
+  <si>
+    <t>um ein Paket zurückzuschicken, melden Sie die Retoure bitte über das Retourenportal in Ihrem Kundenkonto an. Falls Sie als Gast bestellt haben, können Sie die Anmeldung auch mit Ihrer Bestellnummer und Postleitzahl vornehmen</t>
+  </si>
+  <si>
+    <t>K168</t>
+  </si>
+  <si>
+    <t>T-075</t>
+  </si>
+  <si>
+    <t>gilt die gesetzliche Gewährleistung von 2 Jahren ab Lieferung; besteht grundsätzlich noch Anspruch auf Gewährleistung, sofern der Mangel bereits bei Lieferung vorlag oder innerhalb der Gewährleistungsfrist aufgetreten ist</t>
+  </si>
+  <si>
+    <t>Unser Kundenservice wird dann mit Ihnen das weitere Vorgehen besprechen, beispielsweise Reparatur, Ersatz oder andere Lösungen</t>
+  </si>
+  <si>
+    <t>K169</t>
+  </si>
+  <si>
+    <t>T-024</t>
+  </si>
+  <si>
+    <t>eine Lieferung an eine Packstation ist bei der Zahlungsart Kauf auf Rechnung leider nicht möglich, auch wenn der Bestellwert über 49 Euro liegt</t>
+  </si>
+  <si>
+    <t>Das liegt daran, dass die Lieferadresse bei dieser Zahlungsart mit der Rechnungsadresse übereinstimmen muss</t>
+  </si>
+  <si>
+    <t>Bitte beachten Sie, dass bei einer fehlgeschlagenen Kartenzahlung eine 3-D-Secure-Freigabe erforderlich ist und die Bestellung 48 Stunden reserviert bleibt, um die Zahlung erneut durchzuführen</t>
+  </si>
+  <si>
+    <t>K172</t>
+  </si>
+  <si>
+    <t>T-003</t>
+  </si>
+  <si>
+    <t>Die Versandkosten und Lieferzeiten können je nach Produkt und Lieferadresse variieren.</t>
+  </si>
+  <si>
+    <t>K176</t>
+  </si>
+  <si>
+    <t>T-096</t>
+  </si>
+  <si>
+    <t>In der Regel können bei einer verspäteten Zahlung Mahngebühren oder Verzugszinsen anfallen.</t>
+  </si>
+  <si>
+    <t>K188</t>
+  </si>
+  <si>
+    <t>T-002</t>
+  </si>
+  <si>
+    <t>die Lieferung Ihrer Stehlampe als Paket innerhalb Deutschlands dauert in der Regel 2 bis 4 Werktage; Versandkosten betragen 4,95 Euro, sind aber ab einem Bestellwert von 49 Euro versandkostenfrei</t>
+  </si>
+  <si>
+    <t>Expressversand gewählt haben und die Bestellung bis 12 Uhr abgeschlossen sein, erfolgt die Lieferung sogar innerhalb von 1 bis 2 Werktagen, allerdings gegen einen Aufpreis von 9,95 Euro zusätzlich zu den regulären Versandkosten</t>
+  </si>
+  <si>
+    <t>Nach dem Versand erhalten Sie eine Versandbestätigung mit einem Tracking-Link, über den Sie den aktuellen Status Ihrer Lieferung verfolgen können</t>
+  </si>
+  <si>
+    <t>K192</t>
+  </si>
+  <si>
+    <t>T-069</t>
+  </si>
+  <si>
+    <t>für Ersatzteile bei Möbeln der Eigenmarke HD Basics können Sie sich direkt an unseren Kundenservice wenden und dabei die Artikelnummer Ihres Regals angeben.</t>
+  </si>
+  <si>
+    <t>Innerhalb der 5-jährigen Herstellergarantie sind Ersatzteile für HD Basics kostenlos erhältlich, sofern es sich nicht um Bezüge, Polster oder Verschleißteile handelt</t>
+  </si>
+  <si>
+    <t>K195</t>
+  </si>
+  <si>
+    <t>T-006</t>
+  </si>
+  <si>
+    <t>bei einer Lieferung in die Schweiz entstehen für Sie keine zusätzlichen Zoll- oder Einfuhrsteuern bei der Zustellung, da diese bereits im Versandpreis enthalten sind</t>
+  </si>
+  <si>
+    <t>Die Versandkosten für Paketware betragen 14,90 CHF, und es gibt keine Gratisgrenze; Die Lieferzeit beträgt in der Regel 4 bis 8 Werktage</t>
+  </si>
+  <si>
+    <t>Bitte beachten Sie, dass nur Paketware in die Schweiz geliefert werden kann, Speditionsware oder Sperrgut ist für dieses Liefergebiet nicht verfügbar</t>
+  </si>
+  <si>
+    <t>K208</t>
+  </si>
+  <si>
+    <t>Die Kombination von Lieferung an eine Packstation und Zahlung auf Rechnung ist bei uns leider nicht möglich</t>
+  </si>
+  <si>
+    <t>Alternativ können Sie die Lieferung an Ihre Privatadresse wählen und weiterhin auf Rechnung zahlen</t>
+  </si>
+  <si>
+    <t>Eine weitere Möglichkeit ist die Zahlung per Vorkasse oder Kreditkarte, die in Kombination mit der Packstation-Lieferung möglich sind</t>
+  </si>
+  <si>
+    <t>K215</t>
+  </si>
+  <si>
+    <t>T-030</t>
+  </si>
+  <si>
+    <t>Lieferung von Speditionsware erfolgt in der Regel innerhalb von 7–14 Werktagen in Deutschland, wobei die Spedition 1–2 Werktage vor dem Termin anruft und ein Zeitfenster von 4 Stunden vereinbart</t>
+  </si>
+  <si>
+    <t>Eine Lieferung nach 19 Uhr oder am Wochenende können wir leider nicht garantieren, da die genauen Lieferzeiten von der Spedition vorgegeben werden.</t>
+  </si>
+  <si>
+    <t>Falls Sie möchten, können Sie bei der Bestellung die Zusatzleistung „Lieferung in die Wohnung“ buchen. Dabei trägt die Spedition die Ware in den Aufstellraum und nimmt die Verpackung mit</t>
+  </si>
+  <si>
     <t>F1</t>
   </si>
   <si>
-    <t>Fehlerhafte Ware wurde nicht berücksichtigt</t>
-  </si>
-  <si>
-    <t>K074</t>
-  </si>
-  <si>
-    <t>T-040</t>
-  </si>
-  <si>
-    <t>eine Rücksendung ist auch ohne die Originalverpackung möglich, da diese zwar erwünscht, aber nicht verpflichtend ist</t>
-  </si>
-  <si>
-    <t>melden Sie die Rücksendung über das Retourenportal in Ihrem Kundenkonto an oder als Gast mit Bestellnummer und Postleitzahl.</t>
-  </si>
-  <si>
-    <t>Sollte es sich um eine Maßanfertigung handeln, ist eine Rückgabe ausgeschlossen</t>
-  </si>
-  <si>
-    <t>K077</t>
-  </si>
-  <si>
-    <t>T-090</t>
-  </si>
-  <si>
-    <t>Eine Verlängerung der Garantiezeit auf 10 Jahre, auch gegen Aufpreis, ist bei uns derzeit nicht vorgesehen.</t>
-  </si>
-  <si>
-    <t>K078</t>
-  </si>
-  <si>
-    <t>T-011</t>
-  </si>
-  <si>
-    <t>Grundsätzlich bieten wir die Möglichkeit, Lieferungen an Packstationen zu senden, sofern dies vom Versanddienstleister unterstützt wird</t>
-  </si>
-  <si>
-    <t>K088</t>
-  </si>
-  <si>
-    <t>T-067</t>
-  </si>
-  <si>
-    <t>für Möbel der Eigenmarke HD Basics, wie Ihr Regal, erhalten Sie eine 5-Jahres-Herstellergarantie</t>
-  </si>
-  <si>
-    <t>Eine Registrierung des Produkts ist nicht erforderlich. Ihre Rechnung dient als Nachweis für die Garantie</t>
-  </si>
-  <si>
-    <t>K091</t>
-  </si>
-  <si>
-    <t>T-083</t>
-  </si>
-  <si>
-    <t>Bitte melden Sie den Schaden möglichst schnell, idealerweise mit Fotos, damit wir den Fall besser prüfen können. Sie können uns die Fotos gerne per E-Mail oder über das Kontaktformular auf unserer Webseite senden</t>
-  </si>
-  <si>
-    <t>Bezüglich der weiteren Vorgehensweise können wir Ihnen nach Prüfung des Schadens verschiedene Optionen anbieten, wie Ersatzlieferung oder Rückerstattung</t>
-  </si>
-  <si>
-    <t>K099</t>
-  </si>
-  <si>
-    <t>T-104</t>
-  </si>
-  <si>
-    <t>Leider können wir aus Datenschutz- und Sicherheitsgründen keine genauen Gründe für die Ablehnung nennen. Möglicherweise hängt dies mit internen Prüfungen oder Bonitätsbewertungen zusammen.</t>
-  </si>
-  <si>
-    <t>Alternativ bieten wir Ihnen verschiedene andere Zahlungsmöglichkeiten an, wie zum Beispiel Kreditkarte, PayPal oder Vorkasse.</t>
-  </si>
-  <si>
-    <t>K101</t>
-  </si>
-  <si>
-    <t>T-043</t>
-  </si>
-  <si>
-    <t>Rückgabe von Speditionsware in Österreich müssen Sie die Retoure innerhalb von 14 Tagen ab Erhalt der Ware über unseren Kundenservice anmelden</t>
-  </si>
-  <si>
-    <t>vereinbaren Sie bitte einen Abholtermin mit der Spedition. Die Ware muss zerlegt und abholbereit im Erdgeschoss bereitgestellt werden</t>
-  </si>
-  <si>
-    <t>Rücktransportkosten für Speditionsware in Österreich betragen 69 Euro und werden von der Erstattung abgezogen</t>
-  </si>
-  <si>
-    <t>K115</t>
-  </si>
-  <si>
-    <t>K117</t>
-  </si>
-  <si>
-    <t>T-060</t>
-  </si>
-  <si>
-    <t>In der Regel versenden wir Retourenlabels per E-Mail zum Ausdrucken</t>
-  </si>
-  <si>
-    <t>Wenn Sie keinen Drucker zur Verfügung haben, prüfen wir gerne, ob wir Ihnen das Retourenlabel auch per Post zusenden können</t>
-  </si>
-  <si>
-    <t>K123</t>
-  </si>
-  <si>
-    <t>T-042</t>
-  </si>
-  <si>
-    <t>eine Rückgabe von Speditionsware ist grundsätzlich innerhalb von 14 Tagen ab Erhalt möglich; weil 20 Tage nicht mehr möglich</t>
-  </si>
-  <si>
-    <t>Anmeldung einer Rücksendung von Speditionsware ist eine Kontaktaufnahme mit unserem Kundenservice innerhalb der Widerrufsfrist erforderlich. Die Rückgabe erfolgt ausschließlich über den Kundenservice, nicht über das Retourenportal</t>
-  </si>
-  <si>
-    <t>F3</t>
-  </si>
-  <si>
-    <t>Widerruf verstrichen</t>
-  </si>
-  <si>
-    <t>K127</t>
-  </si>
-  <si>
-    <t>T-088</t>
-  </si>
-  <si>
-    <t>K129</t>
-  </si>
-  <si>
-    <t>T-105</t>
-  </si>
-  <si>
-    <t>Grundsätzlich können Geschenkgutscheine von Hallendal Wohnen auch für Bestellungen aus der Schweiz eingelöst werden</t>
-  </si>
-  <si>
-    <t>Bezüglich der Zahlungsmöglichkeiten für Kunden aus der Schweiz bieten wir verschiedene Optionen an</t>
-  </si>
-  <si>
-    <t>K136</t>
-  </si>
-  <si>
-    <t>T-094</t>
-  </si>
-  <si>
-    <t>der Kauf auf Rechnung ist bei Hallendal Wohnen nur bis zu einem maximalen Bestellwert von 1.500 Euro möglich</t>
-  </si>
-  <si>
-    <t>K156</t>
-  </si>
-  <si>
-    <t>Grundsätzlich haben Sie das Recht, Ihre Bestellung innerhalb von 14 Tagen nach Erhalt zurückzugeben.</t>
-  </si>
-  <si>
-    <t>Bezüglich der Erstattung der Versandkosten für den Hinweg hängt dies von den jeweiligen Bedingungen ab, die in unseren Rückgabebedingungen geregelt sind.</t>
-  </si>
-  <si>
-    <t>K159</t>
-  </si>
-  <si>
-    <t>T-080</t>
-  </si>
-  <si>
-    <t>5-Jahres-Herstellergarantie, die ab Lieferung gilt; Das durchgesessene Polster im Kopfteil fällt daher nicht unter die Garantie</t>
-  </si>
-  <si>
-    <t>Für das defekte Teil der Halterung können Sie sich gerne an unseren Kundenservice wenden und die Artikelnummer Ihres Bettes angeben.</t>
-  </si>
-  <si>
-    <t>Montageanleitungen finden Sie als PDF auf der Produktseite Ihres Bettes.</t>
-  </si>
-  <si>
-    <t>K166</t>
-  </si>
-  <si>
-    <t>T-032</t>
-  </si>
-  <si>
-    <t>um ein Paket zurückzuschicken, melden Sie die Retoure bitte über das Retourenportal in Ihrem Kundenkonto an. Falls Sie als Gast bestellt haben, können Sie die Anmeldung auch mit Ihrer Bestellnummer und Postleitzahl vornehmen</t>
-  </si>
-  <si>
-    <t>K168</t>
-  </si>
-  <si>
-    <t>T-075</t>
-  </si>
-  <si>
-    <t>gilt die gesetzliche Gewährleistung von 2 Jahren ab Lieferung; besteht grundsätzlich noch Anspruch auf Gewährleistung, sofern der Mangel bereits bei Lieferung vorlag oder innerhalb der Gewährleistungsfrist aufgetreten ist</t>
-  </si>
-  <si>
-    <t>Unser Kundenservice wird dann mit Ihnen das weitere Vorgehen besprechen, beispielsweise Reparatur, Ersatz oder andere Lösungen</t>
-  </si>
-  <si>
-    <t>K169</t>
-  </si>
-  <si>
-    <t>T-024</t>
-  </si>
-  <si>
-    <t>eine Lieferung an eine Packstation ist bei der Zahlungsart Kauf auf Rechnung leider nicht möglich, auch wenn der Bestellwert über 49 Euro liegt</t>
-  </si>
-  <si>
-    <t>Das liegt daran, dass die Lieferadresse bei dieser Zahlungsart mit der Rechnungsadresse übereinstimmen muss</t>
-  </si>
-  <si>
-    <t>Bitte beachten Sie, dass bei einer fehlgeschlagenen Kartenzahlung eine 3-D-Secure-Freigabe erforderlich ist und die Bestellung 48 Stunden reserviert bleibt, um die Zahlung erneut durchzuführen</t>
-  </si>
-  <si>
-    <t>K172</t>
-  </si>
-  <si>
-    <t>T-003</t>
-  </si>
-  <si>
-    <t>Die Versandkosten und Lieferzeiten können je nach Produkt und Lieferadresse variieren.</t>
-  </si>
-  <si>
-    <t>K176</t>
-  </si>
-  <si>
-    <t>T-096</t>
-  </si>
-  <si>
-    <t>In der Regel können bei einer verspäteten Zahlung Mahngebühren oder Verzugszinsen anfallen.</t>
-  </si>
-  <si>
-    <t>K188</t>
-  </si>
-  <si>
-    <t>T-002</t>
-  </si>
-  <si>
-    <t>die Lieferung Ihrer Stehlampe als Paket innerhalb Deutschlands dauert in der Regel 2 bis 4 Werktage; Versandkosten betragen 4,95 Euro, sind aber ab einem Bestellwert von 49 Euro versandkostenfrei</t>
-  </si>
-  <si>
-    <t>Expressversand gewählt haben und die Bestellung bis 12 Uhr abgeschlossen sein, erfolgt die Lieferung sogar innerhalb von 1 bis 2 Werktagen, allerdings gegen einen Aufpreis von 9,95 Euro zusätzlich zu den regulären Versandkosten</t>
-  </si>
-  <si>
-    <t>Nach dem Versand erhalten Sie eine Versandbestätigung mit einem Tracking-Link, über den Sie den aktuellen Status Ihrer Lieferung verfolgen können</t>
-  </si>
-  <si>
-    <t>K192</t>
-  </si>
-  <si>
-    <t>T-069</t>
-  </si>
-  <si>
-    <t>für Ersatzteile bei Möbeln der Eigenmarke HD Basics können Sie sich direkt an unseren Kundenservice wenden und dabei die Artikelnummer Ihres Regals angeben.</t>
-  </si>
-  <si>
-    <t>Innerhalb der 5-jährigen Herstellergarantie sind Ersatzteile für HD Basics kostenlos erhältlich, sofern es sich nicht um Bezüge, Polster oder Verschleißteile handelt</t>
-  </si>
-  <si>
-    <t>K195</t>
-  </si>
-  <si>
-    <t>T-006</t>
-  </si>
-  <si>
-    <t>bei einer Lieferung in die Schweiz entstehen für Sie keine zusätzlichen Zoll- oder Einfuhrsteuern bei der Zustellung, da diese bereits im Versandpreis enthalten sind</t>
-  </si>
-  <si>
-    <t>Die Versandkosten für Paketware betragen 14,90 CHF, und es gibt keine Gratisgrenze; Die Lieferzeit beträgt in der Regel 4 bis 8 Werktage</t>
-  </si>
-  <si>
-    <t>Bitte beachten Sie, dass nur Paketware in die Schweiz geliefert werden kann, Speditionsware oder Sperrgut ist für dieses Liefergebiet nicht verfügbar</t>
-  </si>
-  <si>
-    <t>K208</t>
-  </si>
-  <si>
-    <t>Die Kombination von Lieferung an eine Packstation und Zahlung auf Rechnung ist bei uns leider nicht möglich</t>
-  </si>
-  <si>
-    <t>Alternativ können Sie die Lieferung an Ihre Privatadresse wählen und weiterhin auf Rechnung zahlen</t>
-  </si>
-  <si>
-    <t>Eine weitere Möglichkeit ist die Zahlung per Vorkasse oder Kreditkarte, die in Kombination mit der Packstation-Lieferung möglich sind</t>
-  </si>
-  <si>
-    <t>K215</t>
-  </si>
-  <si>
-    <t>T-030</t>
-  </si>
-  <si>
-    <t>Lieferung von Speditionsware erfolgt in der Regel innerhalb von 7–14 Werktagen in Deutschland, wobei die Spedition 1–2 Werktage vor dem Termin anruft und ein Zeitfenster von 4 Stunden vereinbart</t>
-  </si>
-  <si>
-    <t>Eine Lieferung nach 19 Uhr oder am Wochenende können wir leider nicht garantieren, da die genauen Lieferzeiten von der Spedition vorgegeben werden.</t>
-  </si>
-  <si>
-    <t>Falls Sie möchten, können Sie bei der Bestellung die Zusatzleistung „Lieferung in die Wohnung“ buchen. Dabei trägt die Spedition die Ware in den Aufstellraum und nimmt die Verpackung mit</t>
+    <t>F3, F4</t>
   </si>
   <si>
     <t>K216</t>
@@ -1073,7 +1076,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>9</v>
@@ -1082,31 +1085,31 @@
         <v>10</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>31</v>
@@ -1115,12 +1118,12 @@
         <v>34</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>40</v>
@@ -1888,21 +1891,21 @@
         <v>56</v>
       </c>
       <c r="P17" s="5" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="Q17" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="S17" s="8" t="s">
         <v>117</v>
-      </c>
-      <c r="S17" s="8" t="s">
-        <v>118</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>120</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>52</v>
@@ -1914,7 +1917,7 @@
         <v>72</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G18" s="5" t="s">
         <v>54</v>
@@ -1923,7 +1926,7 @@
         <v>55</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J18" s="5" t="s">
         <v>54</v>
@@ -1932,7 +1935,7 @@
         <v>55</v>
       </c>
       <c r="L18" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M18" s="5" t="s">
         <v>54</v>
@@ -1953,10 +1956,10 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>124</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>125</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>41</v>
@@ -1968,7 +1971,7 @@
         <v>43</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G19" s="5" t="s">
         <v>54</v>
@@ -1998,10 +2001,10 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>127</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>128</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>41</v>
@@ -2013,7 +2016,7 @@
         <v>72</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G20" s="5" t="s">
         <v>54</v>
@@ -2043,10 +2046,10 @@
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>131</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>52</v>
@@ -2058,7 +2061,7 @@
         <v>72</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G21" s="5" t="s">
         <v>54</v>
@@ -2067,7 +2070,7 @@
         <v>55</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J21" s="5" t="s">
         <v>54</v>
@@ -2091,10 +2094,10 @@
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>134</v>
-      </c>
-      <c r="B22" s="2" t="s">
-        <v>135</v>
       </c>
       <c r="C22" s="2" t="s">
         <v>41</v>
@@ -2106,7 +2109,7 @@
         <v>66</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G22" s="5" t="s">
         <v>54</v>
@@ -2115,7 +2118,7 @@
         <v>46</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J22" s="5" t="s">
         <v>54</v>
@@ -2142,10 +2145,10 @@
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>139</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>41</v>
@@ -2157,7 +2160,7 @@
         <v>60</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G23" s="5" t="s">
         <v>45</v>
@@ -2166,7 +2169,7 @@
         <v>46</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="J23" s="5" t="s">
         <v>45</v>
@@ -2193,10 +2196,10 @@
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>143</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>52</v>
@@ -2208,7 +2211,7 @@
         <v>60</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G24" s="5" t="s">
         <v>54</v>
@@ -2217,7 +2220,7 @@
         <v>55</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="J24" s="5" t="s">
         <v>54</v>
@@ -2226,12 +2229,14 @@
         <v>55</v>
       </c>
       <c r="L24" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="M24" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="N24" s="2"/>
+      <c r="N24" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="O24" s="5" t="s">
         <v>56</v>
       </c>
@@ -2245,7 +2250,7 @@
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>107</v>
@@ -2268,7 +2273,9 @@
       <c r="L25" s="4"/>
       <c r="M25" s="2"/>
       <c r="N25" s="6"/>
-      <c r="O25" s="2"/>
+      <c r="O25" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="P25" s="6" t="s">
         <v>49</v>
       </c>
@@ -2282,10 +2289,10 @@
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>149</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>41</v>
@@ -2297,7 +2304,7 @@
         <v>43</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G26" s="5" t="s">
         <v>54</v>
@@ -2306,7 +2313,7 @@
         <v>46</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="J26" s="5" t="s">
         <v>74</v>
@@ -2333,10 +2340,10 @@
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>153</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>52</v>
@@ -2348,7 +2355,7 @@
         <v>60</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G27" s="5" t="s">
         <v>54</v>
@@ -2357,7 +2364,7 @@
         <v>55</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>54</v>
@@ -2375,18 +2382,18 @@
         <v>48</v>
       </c>
       <c r="Q27" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="S27" s="8" t="s">
         <v>156</v>
-      </c>
-      <c r="S27" s="8" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="B28" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>41</v>
@@ -2406,7 +2413,9 @@
       <c r="L28" s="4"/>
       <c r="M28" s="2"/>
       <c r="N28" s="6"/>
-      <c r="O28" s="2"/>
+      <c r="O28" s="5" t="s">
+        <v>48</v>
+      </c>
       <c r="P28" s="6" t="s">
         <v>49</v>
       </c>
@@ -2420,10 +2429,10 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>161</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>41</v>
@@ -2435,7 +2444,7 @@
         <v>60</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G29" s="5" t="s">
         <v>54</v>
@@ -2444,7 +2453,7 @@
         <v>46</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J29" s="5" t="s">
         <v>54</v>
@@ -2471,10 +2480,10 @@
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>164</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>165</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>52</v>
@@ -2486,7 +2495,7 @@
         <v>72</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G30" s="5" t="s">
         <v>54</v>
@@ -2513,7 +2522,7 @@
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>59</v>
@@ -2528,7 +2537,7 @@
         <v>60</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G31" s="5" t="s">
         <v>54</v>
@@ -2537,7 +2546,7 @@
         <v>46</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>45</v>
@@ -2564,10 +2573,10 @@
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>170</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>171</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>52</v>
@@ -2579,7 +2588,7 @@
         <v>66</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G32" s="5" t="s">
         <v>54</v>
@@ -2588,16 +2597,16 @@
         <v>55</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="J32" s="5" t="s">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="K32" s="5" t="s">
         <v>55</v>
       </c>
       <c r="L32" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="M32" s="5" t="s">
         <v>54</v>
@@ -2618,10 +2627,10 @@
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>175</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>176</v>
       </c>
       <c r="C33" s="2" t="s">
         <v>52</v>
@@ -2633,7 +2642,7 @@
         <v>72</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G33" s="5" t="s">
         <v>54</v>
@@ -2660,10 +2669,10 @@
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="B34" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>52</v>
@@ -2675,7 +2684,7 @@
         <v>60</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G34" s="5" t="s">
         <v>54</v>
@@ -2684,7 +2693,7 @@
         <v>55</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="J34" s="5" t="s">
         <v>54</v>
@@ -2708,10 +2717,10 @@
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>182</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>183</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>52</v>
@@ -2723,7 +2732,7 @@
         <v>66</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G35" s="5" t="s">
         <v>54</v>
@@ -2732,7 +2741,7 @@
         <v>55</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="J35" s="5" t="s">
         <v>54</v>
@@ -2741,12 +2750,14 @@
         <v>55</v>
       </c>
       <c r="L35" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="M35" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="N35" s="2"/>
+      <c r="N35" s="5" t="s">
+        <v>55</v>
+      </c>
       <c r="O35" s="5" t="s">
         <v>56</v>
       </c>
@@ -2760,10 +2771,10 @@
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>187</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>188</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>41</v>
@@ -2775,7 +2786,7 @@
         <v>72</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G36" s="5" t="s">
         <v>45</v>
@@ -2805,10 +2816,10 @@
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>190</v>
-      </c>
-      <c r="B37" s="2" t="s">
-        <v>191</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>41</v>
@@ -2820,7 +2831,7 @@
         <v>72</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G37" s="5" t="s">
         <v>74</v>
@@ -2850,10 +2861,10 @@
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>193</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>194</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>52</v>
@@ -2865,7 +2876,7 @@
         <v>72</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G38" s="5" t="s">
         <v>54</v>
@@ -2874,7 +2885,7 @@
         <v>55</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J38" s="5" t="s">
         <v>54</v>
@@ -2883,7 +2894,7 @@
         <v>55</v>
       </c>
       <c r="L38" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="M38" s="5" t="s">
         <v>54</v>
@@ -2904,10 +2915,10 @@
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>198</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>199</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>52</v>
@@ -2919,7 +2930,7 @@
         <v>72</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G39" s="5" t="s">
         <v>54</v>
@@ -2928,7 +2939,7 @@
         <v>55</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="J39" s="5" t="s">
         <v>54</v>
@@ -2952,10 +2963,10 @@
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>202</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>203</v>
       </c>
       <c r="C40" s="2" t="s">
         <v>52</v>
@@ -2967,7 +2978,7 @@
         <v>72</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G40" s="5" t="s">
         <v>54</v>
@@ -2976,7 +2987,7 @@
         <v>55</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="J40" s="5" t="s">
         <v>54</v>
@@ -2985,7 +2996,7 @@
         <v>55</v>
       </c>
       <c r="L40" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="M40" s="5" t="s">
         <v>54</v>
@@ -3006,10 +3017,10 @@
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="3" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>41</v>
@@ -3021,7 +3032,7 @@
         <v>66</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G41" s="5" t="s">
         <v>54</v>
@@ -3030,7 +3041,7 @@
         <v>46</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="J41" s="5" t="s">
         <v>54</v>
@@ -3039,7 +3050,7 @@
         <v>46</v>
       </c>
       <c r="L41" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M41" s="5" t="s">
         <v>54</v>
@@ -3063,10 +3074,10 @@
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>211</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>212</v>
       </c>
       <c r="C42" s="2" t="s">
         <v>52</v>
@@ -3078,7 +3089,7 @@
         <v>43</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G42" s="5" t="s">
         <v>54</v>
@@ -3087,7 +3098,7 @@
         <v>55</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J42" s="5" t="s">
         <v>45</v>
@@ -3096,7 +3107,7 @@
         <v>46</v>
       </c>
       <c r="L42" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="M42" s="5" t="s">
         <v>54</v>
@@ -3108,19 +3119,22 @@
         <v>56</v>
       </c>
       <c r="P42" s="5" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="Q42" s="5" t="s">
-        <v>57</v>
+        <v>215</v>
+      </c>
+      <c r="R42" s="5" t="s">
+        <v>216</v>
       </c>
       <c r="S42" s="7"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C43" s="2" t="s">
         <v>41</v>
@@ -3132,7 +3146,7 @@
         <v>60</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G43" s="5" t="s">
         <v>45</v>
@@ -3141,7 +3155,7 @@
         <v>46</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J43" s="5" t="s">
         <v>74</v>
@@ -3168,7 +3182,7 @@
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>87</v>
@@ -3183,7 +3197,7 @@
         <v>66</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G44" s="5" t="s">
         <v>74</v>
@@ -3213,10 +3227,10 @@
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C45" s="2" t="s">
         <v>41</v>
@@ -3228,7 +3242,7 @@
         <v>60</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G45" s="5" t="s">
         <v>54</v>
@@ -3237,7 +3251,7 @@
         <v>46</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J45" s="5" t="s">
         <v>54</v>
@@ -3264,10 +3278,10 @@
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C46" s="2" t="s">
         <v>52</v>
@@ -3279,7 +3293,7 @@
         <v>72</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G46" s="5" t="s">
         <v>54</v>
@@ -3288,7 +3302,7 @@
         <v>55</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J46" s="5" t="s">
         <v>54</v>
@@ -3297,7 +3311,7 @@
         <v>55</v>
       </c>
       <c r="L46" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="M46" s="5" t="s">
         <v>54</v>
@@ -3308,16 +3322,20 @@
       <c r="O46" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="P46" s="2"/>
-      <c r="Q46" s="2"/>
+      <c r="P46" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q46" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="S46" s="7"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>52</v>
@@ -3329,7 +3347,7 @@
         <v>72</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G47" s="5" t="s">
         <v>54</v>
@@ -3338,7 +3356,7 @@
         <v>55</v>
       </c>
       <c r="I47" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="J47" s="5" t="s">
         <v>54</v>
@@ -3347,7 +3365,7 @@
         <v>55</v>
       </c>
       <c r="L47" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="M47" s="5" t="s">
         <v>54</v>
@@ -3358,16 +3376,20 @@
       <c r="O47" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="P47" s="2"/>
-      <c r="Q47" s="2"/>
+      <c r="P47" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q47" s="5" t="s">
+        <v>57</v>
+      </c>
       <c r="S47" s="7"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>41</v>
@@ -3379,7 +3401,7 @@
         <v>43</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G48" s="5" t="s">
         <v>54</v>
@@ -3409,10 +3431,10 @@
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C49" s="2" t="s">
         <v>41</v>
@@ -3424,7 +3446,7 @@
         <v>43</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G49" s="5" t="s">
         <v>45</v>
@@ -4501,57 +4523,57 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="C3" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -4573,18 +4595,18 @@
         <v>35</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>